<commit_message>
fix dataset & extract model pathes
</commit_message>
<xml_diff>
--- a/backend/data/processed/cleaned_hospital_data.xlsx
+++ b/backend/data/processed/cleaned_hospital_data.xlsx
@@ -881,10 +881,10 @@
         <v>79.5</v>
       </c>
       <c r="F11" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G11" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H11" t="n">
         <v>4</v>
@@ -1212,7 +1212,7 @@
         <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
@@ -1253,7 +1253,7 @@
         <v>9</v>
       </c>
       <c r="G20" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H20" t="n">
         <v>1</v>
@@ -1581,7 +1581,7 @@
         <v>5</v>
       </c>
       <c r="G28" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H28" t="n">
         <v>5</v>
@@ -1622,7 +1622,7 @@
         <v>8</v>
       </c>
       <c r="G29" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H29" t="n">
         <v>2</v>
@@ -1824,10 +1824,10 @@
         <v>79.5</v>
       </c>
       <c r="F34" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G34" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H34" t="n">
         <v>5</v>
@@ -2521,10 +2521,10 @@
         <v>81</v>
       </c>
       <c r="F51" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G51" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H51" t="n">
         <v>5</v>
@@ -2770,7 +2770,7 @@
         <v>3</v>
       </c>
       <c r="G57" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H57" t="n">
         <v>5</v>
@@ -3262,7 +3262,7 @@
         <v>9</v>
       </c>
       <c r="G69" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H69" t="n">
         <v>1</v>
@@ -3754,7 +3754,7 @@
         <v>5</v>
       </c>
       <c r="G81" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H81" t="n">
         <v>5</v>
@@ -4000,7 +4000,7 @@
         <v>6</v>
       </c>
       <c r="G87" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H87" t="n">
         <v>3</v>
@@ -4410,7 +4410,7 @@
         <v>8</v>
       </c>
       <c r="G97" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H97" t="n">
         <v>3</v>
@@ -4940,7 +4940,7 @@
         <v>79.5</v>
       </c>
       <c r="F110" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G110" t="n">
         <v>18</v>
@@ -5066,7 +5066,7 @@
         <v>3</v>
       </c>
       <c r="G113" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H113" t="n">
         <v>5</v>
@@ -6009,7 +6009,7 @@
         <v>3</v>
       </c>
       <c r="G136" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H136" t="n">
         <v>2</v>
@@ -6744,7 +6744,7 @@
         <v>79.5</v>
       </c>
       <c r="F154" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G154" t="n">
         <v>21</v>
@@ -6952,7 +6952,7 @@
         <v>9</v>
       </c>
       <c r="G159" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H159" t="n">
         <v>3</v>
@@ -7113,7 +7113,7 @@
         <v>79.5</v>
       </c>
       <c r="F163" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G163" t="n">
         <v>12</v>
@@ -7321,7 +7321,7 @@
         <v>5</v>
       </c>
       <c r="G168" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H168" t="n">
         <v>4</v>
@@ -7854,7 +7854,7 @@
         <v>7</v>
       </c>
       <c r="G181" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H181" t="n">
         <v>5</v>
@@ -8674,7 +8674,7 @@
         <v>9</v>
       </c>
       <c r="G201" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H201" t="n">
         <v>4</v>
@@ -9207,7 +9207,7 @@
         <v>7</v>
       </c>
       <c r="G214" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H214" t="n">
         <v>2</v>
@@ -9289,7 +9289,7 @@
         <v>3</v>
       </c>
       <c r="G216" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H216" t="n">
         <v>4</v>
@@ -10273,7 +10273,7 @@
         <v>6</v>
       </c>
       <c r="G240" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H240" t="n">
         <v>2</v>
@@ -10639,10 +10639,10 @@
         <v>79.5</v>
       </c>
       <c r="F249" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G249" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H249" t="n">
         <v>4</v>
@@ -10724,7 +10724,7 @@
         <v>5</v>
       </c>
       <c r="G251" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H251" t="n">
         <v>5</v>
@@ -10967,7 +10967,7 @@
         <v>85</v>
       </c>
       <c r="F257" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G257" t="n">
         <v>17</v>
@@ -11869,10 +11869,10 @@
         <v>79.5</v>
       </c>
       <c r="F279" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G279" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H279" t="n">
         <v>4</v>
@@ -12651,7 +12651,7 @@
         <v>5</v>
       </c>
       <c r="G298" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H298" t="n">
         <v>4</v>
@@ -12856,7 +12856,7 @@
         <v>8</v>
       </c>
       <c r="G303" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H303" t="n">
         <v>5</v>
@@ -12894,10 +12894,10 @@
         <v>79.5</v>
       </c>
       <c r="F304" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G304" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H304" t="n">
         <v>3</v>
@@ -13222,7 +13222,7 @@
         <v>79.5</v>
       </c>
       <c r="F312" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G312" t="n">
         <v>19</v>
@@ -14165,7 +14165,7 @@
         <v>91</v>
       </c>
       <c r="F335" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G335" t="n">
         <v>7</v>
@@ -14329,7 +14329,7 @@
         <v>79.5</v>
       </c>
       <c r="F339" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G339" t="n">
         <v>13</v>
@@ -14657,10 +14657,10 @@
         <v>90</v>
       </c>
       <c r="F347" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G347" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H347" t="n">
         <v>5</v>
@@ -15357,7 +15357,7 @@
         <v>5</v>
       </c>
       <c r="G364" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H364" t="n">
         <v>3</v>
@@ -17691,10 +17691,10 @@
         <v>79.5</v>
       </c>
       <c r="F421" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G421" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H421" t="n">
         <v>4</v>
@@ -17773,10 +17773,10 @@
         <v>79.5</v>
       </c>
       <c r="F423" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G423" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H423" t="n">
         <v>5</v>
@@ -18391,7 +18391,7 @@
         <v>7</v>
       </c>
       <c r="G438" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H438" t="n">
         <v>5</v>
@@ -19208,7 +19208,7 @@
         <v>94</v>
       </c>
       <c r="F458" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G458" t="n">
         <v>21</v>
@@ -19293,7 +19293,7 @@
         <v>9</v>
       </c>
       <c r="G460" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H460" t="n">
         <v>3</v>
@@ -19867,7 +19867,7 @@
         <v>9</v>
       </c>
       <c r="G474" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H474" t="n">
         <v>3</v>
@@ -20810,7 +20810,7 @@
         <v>7</v>
       </c>
       <c r="G497" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H497" t="n">
         <v>1</v>
@@ -20889,10 +20889,10 @@
         <v>79.5</v>
       </c>
       <c r="F499" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G499" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H499" t="n">
         <v>2</v>
@@ -22119,10 +22119,10 @@
         <v>79.5</v>
       </c>
       <c r="F529" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G529" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H529" t="n">
         <v>5</v>
@@ -22450,7 +22450,7 @@
         <v>9</v>
       </c>
       <c r="G537" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H537" t="n">
         <v>4</v>
@@ -22611,7 +22611,7 @@
         <v>79.5</v>
       </c>
       <c r="F541" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G541" t="n">
         <v>23</v>
@@ -22696,7 +22696,7 @@
         <v>7</v>
       </c>
       <c r="G543" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H543" t="n">
         <v>5</v>
@@ -22778,7 +22778,7 @@
         <v>6</v>
       </c>
       <c r="G545" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H545" t="n">
         <v>1</v>
@@ -22857,7 +22857,7 @@
         <v>79.5</v>
       </c>
       <c r="F547" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="G547" t="n">
         <v>10</v>
@@ -23311,7 +23311,7 @@
         <v>3</v>
       </c>
       <c r="G558" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H558" t="n">
         <v>5</v>
@@ -23516,7 +23516,7 @@
         <v>5</v>
       </c>
       <c r="G563" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H563" t="n">
         <v>5</v>
@@ -23557,7 +23557,7 @@
         <v>9</v>
       </c>
       <c r="G564" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H564" t="n">
         <v>2</v>
@@ -23926,7 +23926,7 @@
         <v>8</v>
       </c>
       <c r="G573" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H573" t="n">
         <v>5</v>
@@ -24213,7 +24213,7 @@
         <v>6</v>
       </c>
       <c r="G580" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H580" t="n">
         <v>3</v>
@@ -24582,7 +24582,7 @@
         <v>9</v>
       </c>
       <c r="G589" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H589" t="n">
         <v>3</v>
@@ -24992,7 +24992,7 @@
         <v>3</v>
       </c>
       <c r="G599" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H599" t="n">
         <v>4</v>
@@ -26509,7 +26509,7 @@
         <v>8</v>
       </c>
       <c r="G636" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H636" t="n">
         <v>4</v>
@@ -26591,7 +26591,7 @@
         <v>9</v>
       </c>
       <c r="G638" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="H638" t="n">
         <v>4</v>

</xml_diff>